<commit_message>
docs: 2026-08-31 — add speed-audit CSVs (Jefri Req1-8, all-staff table) as tabs in the requirement usage workbook, sourced from earlier session's live timing tests
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNdpYHXbhVyvHRUcdfXbv2
</commit_message>
<xml_diff>
--- a/prompts/team-usage-csv/Team_Requirement_Usage_AllTabs.xlsx
+++ b/prompts/team-usage-csv/Team_Requirement_Usage_AllTabs.xlsx
@@ -18,6 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theekshy" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hetheesha" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thivajini" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speed - Jefri" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speed - All Staff" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -970,6 +972,1157 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Req 1 - Product Status Labels</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>16.97s</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>14.49s</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>~15.7s</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Req 2 - Search Terms Labels</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>7.36s</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7.39s</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>~7.4s</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Req 3 - 3-Period Comparison</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>5.02s</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3.11s</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>~4.1s</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Req 4 - Item ID -&gt; Parent Mapping</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4.05s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2.72s</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>~3.4s</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Req 5 - Cross-Campaign Attribution</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3.22s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1.91s</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>~2.6s</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Req 6 - Image Update Tracker</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>11.86s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>11.95s</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>~11.9s</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Req 7 - SKU &amp; Price Reconciliation</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1.39s</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1.46s</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>~1.4s</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Req 8 - Order Conversion Split</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>18.35s</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>12.10s</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>~15.2s</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Hetheesha</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Req 5 - Internal Link Audit</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>143.97s</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Critical - worst in the app</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hetheesha</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Req 4 - High-Traffic Stock Alert</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>68.02s</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hetheesha</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Req 3 - Duplicate Page Analysis</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>46.50s</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dilaksi</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Req 1 - GA4 SEO Performance</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>25.86s</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Kamsi</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Req 3 - GA4 SEO Performance</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>25.43s</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mahima</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Req 1 - Product Performance Report</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>20.09s</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hetheesha</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Req 1 - Product SEO Report</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>18.51s</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kamsi</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Req 2 - Low CTR Pages</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>15.86s</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mahima</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Req 5 - Product ID Coverage</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>15.80s</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Thasitha</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Req 2 - PMax Zero-Performance</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15.36s</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thasitha</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Req 7 - Amazon DE Search Terms</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>13.35s</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Very slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Thivajini</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Req 1 - Conversion Tracking</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>12.74s</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Mahima</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Search Terms</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7.08s</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sukirtha</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Req 4 - GA4 SEO Performance</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>6.31s</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Thasitha</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Req 6 - Search Terms Labels</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5.20s</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sonya</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Product Performance</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>5.40s</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sonya</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Trend &amp; Segment Dashboard</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>4.78s</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sukirtha</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Req 1 - Low CTR Blog/Collections</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4.88s</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sonya</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Opportunity Tab</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4.14s</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sajeepan</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Req 3 - Product Action Dashboard</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>3.82s</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hetheesha</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Req 2 - Collection Performance</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>3.83s</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Thivajini</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Req 3 - Stock-Spend Tracker</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3.80s</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thivajini</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Req 4 - Order Data</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>3.78s</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sajeepan</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Req 2 - Revenue Protection</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>3.46s</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Sonya</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Stop Waste Spend</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2.84s</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sonya</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Daily Orders</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2.78s</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sajeepan</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Req 1 - Product Intelligence</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2.76s</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sajeepan</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Req 4 - Feed Optimization</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2.70s</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Thivajini</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Req 2 - Product-Level Performance</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2.85s</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Theekshy</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Req 5 - Product Optimisation</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2.56s</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Theekshy</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Req 1 - Campaign Optimisation</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2.01s</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Theekshy</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Req 3 - Feed Optimisation</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2.06s</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Theekshy</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Req 4 - Stock Status Snapshot</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1.87s</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Theekshy</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Req 2 - Search Term Optimisation</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1.23s</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Thasitha</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Req 1 - Campaign Performance</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1.16s</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sonya</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Campaign Performance</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>0.96s</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Dilaksi</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Req 3 - Collections Removal Audit</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>0.38s</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Thasitha</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Req 3 - Item ID Cross-Campaign</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>0.35s</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Kamsi Req1/4/5/6; Mahima Req2/5b; Dilaksi Req2; Sukirtha Req2/3/5/6; Thasitha Req4/5</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>~0.2s each</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Already fast</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>